<commit_message>
minor update in main branch
</commit_message>
<xml_diff>
--- a/portfolio_summary.xlsx
+++ b/portfolio_summary.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kalongli\Desktop\Git\portfolio_rebalance\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{40688654-E2C3-4C64-8950-93F5868F3BDB}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A0A7ACF0-0996-4A35-98A5-E6C06418B448}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,29 +25,9 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1" uniqueCount="1">
   <si>
     <t>Rebalancing_date</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>VT</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>TQQQ</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>CASH</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>QQQ</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>MQQQ</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -91,9 +71,8 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -374,37 +353,20 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F2"/>
+  <dimension ref="A1"/>
   <sheetFormatPr defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="16.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1" t="s">
-        <v>4</v>
-      </c>
-      <c r="F1" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A2" s="1"/>
     </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
add gen report function
</commit_message>
<xml_diff>
--- a/portfolio_summary.xlsx
+++ b/portfolio_summary.xlsx
@@ -8,12 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kalongli\Desktop\Git\portfolio_rebalance\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{40688654-E2C3-4C64-8950-93F5868F3BDB}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3F6543C3-C30E-4CF3-A2C2-7F9C603C5E0C}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="rebalancing_overview" sheetId="1" r:id="rId1"/>
+    <sheet name="performance" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -25,29 +26,9 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1" uniqueCount="1">
   <si>
     <t>Rebalancing_date</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>VT</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>TQQQ</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>CASH</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>QQQ</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>MQQQ</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -374,37 +355,33 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F2"/>
+  <dimension ref="A1:A2"/>
   <sheetFormatPr defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="16.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1" t="s">
-        <v>4</v>
-      </c>
-      <c r="F1" t="s">
-        <v>5</v>
-      </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" s="1"/>
     </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C035171E-080D-4182-8FEE-61627FF839E3}">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
+  <sheetData/>
+  <phoneticPr fontId="1" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
change the message to no. of shs instead of the amount needed to buy/sell
</commit_message>
<xml_diff>
--- a/portfolio_summary.xlsx
+++ b/portfolio_summary.xlsx
@@ -1,38 +1,91 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28925"/>
   <workbookPr/>
-  <workbookProtection/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Antho\OneDrive\Desktop\Git\portfolio_rebalance\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D655F58B-700E-4A54-8215-062E5B116DEC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="rebalancing_overview" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Performance" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="rebalancing_overview" sheetId="1" r:id="rId1"/>
+    <sheet name="Performance" sheetId="2" r:id="rId2"/>
   </sheets>
-  <definedNames/>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="14">
+  <si>
+    <t>Rebalance_Date</t>
+  </si>
+  <si>
+    <t>AVDV</t>
+  </si>
+  <si>
+    <t>AVUV</t>
+  </si>
+  <si>
+    <t>CASH</t>
+  </si>
+  <si>
+    <t>SGOV</t>
+  </si>
+  <si>
+    <t>SQQQ</t>
+  </si>
+  <si>
+    <t>VT</t>
+  </si>
+  <si>
+    <t>2025-07-31</t>
+  </si>
+  <si>
+    <t>2.00% (+0.00%)</t>
+  </si>
+  <si>
+    <t>4.50% (+0.00%)</t>
+  </si>
+  <si>
+    <t>4.93% (+0.00%)</t>
+  </si>
+  <si>
+    <t>65.07% (+0.00%)</t>
+  </si>
+  <si>
+    <t>1.00% (+0.00%)</t>
+  </si>
+  <si>
+    <t>22.50% (+0.00%)</t>
+  </si>
+</sst>
+</file>
+
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
-  <fonts count="2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
-      <color theme="1"/>
-      <sz val="11"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <b val="1"/>
+      <b/>
+      <sz val="11"/>
+      <name val="Calibri"/>
     </font>
   </fonts>
   <fills count="2">
     <fill>
-      <patternFill/>
+      <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
@@ -47,93 +100,43 @@
       <diagonal/>
     </border>
     <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
     </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="2">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
+  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
-  <colors>
-    <indexedColors>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008000"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00808000"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="00C0C0C0"/>
-      <rgbColor rgb="00808080"/>
-      <rgbColor rgb="009999FF"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00FFFFCC"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00660066"/>
-      <rgbColor rgb="00FF8080"/>
-      <rgbColor rgb="000066CC"/>
-      <rgbColor rgb="00CCCCFF"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="0000CCFF"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00CCFFCC"/>
-      <rgbColor rgb="00FFFF99"/>
-      <rgbColor rgb="0099CCFF"/>
-      <rgbColor rgb="00FF99CC"/>
-      <rgbColor rgb="00CC99FF"/>
-      <rgbColor rgb="00FFCC99"/>
-      <rgbColor rgb="003366FF"/>
-      <rgbColor rgb="0033CCCC"/>
-      <rgbColor rgb="0099CC00"/>
-      <rgbColor rgb="00FFCC00"/>
-      <rgbColor rgb="00FF9900"/>
-      <rgbColor rgb="00FF6600"/>
-      <rgbColor rgb="00666699"/>
-      <rgbColor rgb="00969696"/>
-      <rgbColor rgb="00003366"/>
-      <rgbColor rgb="00339966"/>
-      <rgbColor rgb="00003300"/>
-      <rgbColor rgb="00333300"/>
-      <rgbColor rgb="00993300"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00333399"/>
-      <rgbColor rgb="00333333"/>
-    </indexedColors>
-  </colors>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
@@ -421,86 +424,61 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:G2"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="15.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="4" width="14.28515625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="15.28515625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="14.28515625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="15.28515625" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Rebalance_Date</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>AVDV</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>AVUV</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>CASH</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>SQQQ</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>US-T</t>
-        </is>
-      </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>VT</t>
-        </is>
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>6</v>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>2025-07-31</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>2.00% (+0.00%)</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>4.50% (+0.00%)</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>0.00% (+0.00%)</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>1.00% (+0.00%)</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>70.00% (+0.00%)</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>22.50% (+0.00%)</t>
-        </is>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>7</v>
+      </c>
+      <c r="B2" t="s">
+        <v>8</v>
+      </c>
+      <c r="C2" t="s">
+        <v>9</v>
+      </c>
+      <c r="D2" t="s">
+        <v>10</v>
+      </c>
+      <c r="E2" t="s">
+        <v>11</v>
+      </c>
+      <c r="F2" t="s">
+        <v>12</v>
+      </c>
+      <c r="G2" t="s">
+        <v>13</v>
       </c>
     </row>
   </sheetData>
@@ -509,13 +487,9 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:A1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
add UI function intergrating with IBKR
</commit_message>
<xml_diff>
--- a/portfolio_summary.xlsx
+++ b/portfolio_summary.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Antho\OneDrive\Desktop\Git\portfolio_rebalance\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D655F58B-700E-4A54-8215-062E5B116DEC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{264DDEE0-6394-4A78-A5AC-429EA7C3E964}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="9075" yWindow="3480" windowWidth="14340" windowHeight="11475" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="rebalancing_overview" sheetId="1" r:id="rId1"/>
@@ -427,13 +427,6 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:G2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="1" width="15.42578125" bestFit="1" customWidth="1"/>
-    <col min="2" max="4" width="14.28515625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="15.28515625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="14.28515625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="15.28515625" bestFit="1" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
@@ -490,7 +483,9 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData/>
+  <sheetData>
+    <row r="1" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
+  </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
add the function for modifying the ratio in UI
</commit_message>
<xml_diff>
--- a/portfolio_summary.xlsx
+++ b/portfolio_summary.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Antho\OneDrive\Desktop\Git\portfolio_rebalance\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1C28948A-0835-4B61-B033-ADEAB8BA7D45}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5C3AF10B-19BE-42D6-AB38-FFE1ED91CA58}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -490,7 +490,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="3" spans="1:7" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>14</v>
       </c>

</xml_diff>

<commit_message>
update the calculation logic for tradable fund
</commit_message>
<xml_diff>
--- a/portfolio_summary.xlsx
+++ b/portfolio_summary.xlsx
@@ -1,100 +1,38 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29029"/>
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Antho\OneDrive\Desktop\Git\portfolio_rebalance\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5C3AF10B-19BE-42D6-AB38-FFE1ED91CA58}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <workbookProtection/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="rebalancing_overview" sheetId="1" r:id="rId1"/>
-    <sheet name="Performance" sheetId="2" r:id="rId2"/>
+    <sheet name="rebalancing_overview" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Performance" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <definedNames/>
+  <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
-<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="17">
-  <si>
-    <t>Rebalance_Date</t>
-  </si>
-  <si>
-    <t>AVDV</t>
-  </si>
-  <si>
-    <t>AVUV</t>
-  </si>
-  <si>
-    <t>CASH</t>
-  </si>
-  <si>
-    <t>SGOV</t>
-  </si>
-  <si>
-    <t>SQQQ</t>
-  </si>
-  <si>
-    <t>VT</t>
-  </si>
-  <si>
-    <t>2025-07-31</t>
-  </si>
-  <si>
-    <t>2.00% (+0.00%)</t>
-  </si>
-  <si>
-    <t>4.50% (+0.00%)</t>
-  </si>
-  <si>
-    <t>4.93% (+0.00%)</t>
-  </si>
-  <si>
-    <t>65.07% (+0.00%)</t>
-  </si>
-  <si>
-    <t>1.00% (+0.00%)</t>
-  </si>
-  <si>
-    <t>22.50% (+0.00%)</t>
-  </si>
-  <si>
-    <t>2025-08-04</t>
-  </si>
-  <si>
-    <t>0.00% (-4.93%)</t>
-  </si>
-  <si>
-    <t>70.00% (+4.93%)</t>
-  </si>
-</sst>
-</file>
-
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <numFmts count="0"/>
+  <fonts count="2">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
+      <color theme="1"/>
+      <sz val="11"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <b/>
-      <sz val="11"/>
-      <name val="Calibri"/>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
     <fill>
-      <patternFill patternType="none"/>
+      <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
@@ -109,43 +47,93 @@
       <diagonal/>
     </border>
     <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
     </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="2">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
   </cellStyles>
-  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
+  <colors>
+    <indexedColors>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008000"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00808000"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="00C0C0C0"/>
+      <rgbColor rgb="00808080"/>
+      <rgbColor rgb="009999FF"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00FFFFCC"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00660066"/>
+      <rgbColor rgb="00FF8080"/>
+      <rgbColor rgb="000066CC"/>
+      <rgbColor rgb="00CCCCFF"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="0000CCFF"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00CCFFCC"/>
+      <rgbColor rgb="00FFFF99"/>
+      <rgbColor rgb="0099CCFF"/>
+      <rgbColor rgb="00FF99CC"/>
+      <rgbColor rgb="00CC99FF"/>
+      <rgbColor rgb="00FFCC99"/>
+      <rgbColor rgb="003366FF"/>
+      <rgbColor rgb="0033CCCC"/>
+      <rgbColor rgb="0099CC00"/>
+      <rgbColor rgb="00FFCC00"/>
+      <rgbColor rgb="00FF9900"/>
+      <rgbColor rgb="00FF6600"/>
+      <rgbColor rgb="00666699"/>
+      <rgbColor rgb="00969696"/>
+      <rgbColor rgb="00003366"/>
+      <rgbColor rgb="00339966"/>
+      <rgbColor rgb="00003300"/>
+      <rgbColor rgb="00333300"/>
+      <rgbColor rgb="00993300"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00333399"/>
+      <rgbColor rgb="00333333"/>
+    </indexedColors>
+  </colors>
 </styleSheet>
 </file>
 
@@ -433,84 +421,160 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G3"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="1" width="15.42578125" bestFit="1" customWidth="1"/>
-    <col min="2" max="4" width="14.28515625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="15.28515625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="14.28515625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="15.28515625" bestFit="1" customWidth="1"/>
-  </cols>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>6</v>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Rebalance_Date</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>AVDV</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>AVUV</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>CASH</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>SGOV</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>SQQQ</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>VT</t>
+        </is>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>7</v>
-      </c>
-      <c r="B2" t="s">
-        <v>8</v>
-      </c>
-      <c r="C2" t="s">
-        <v>9</v>
-      </c>
-      <c r="D2" t="s">
-        <v>10</v>
-      </c>
-      <c r="E2" t="s">
-        <v>11</v>
-      </c>
-      <c r="F2" t="s">
-        <v>12</v>
-      </c>
-      <c r="G2" t="s">
-        <v>13</v>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>2025-07-31</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>2.00% (+0.00%)</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>4.50% (+0.00%)</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>4.93% (+0.00%)</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>65.07% (+0.00%)</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>1.00% (+0.00%)</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>22.50% (+0.00%)</t>
+        </is>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>14</v>
-      </c>
-      <c r="B3" t="s">
-        <v>8</v>
-      </c>
-      <c r="C3" t="s">
-        <v>9</v>
-      </c>
-      <c r="D3" t="s">
-        <v>15</v>
-      </c>
-      <c r="E3" t="s">
-        <v>16</v>
-      </c>
-      <c r="F3" t="s">
-        <v>12</v>
-      </c>
-      <c r="G3" t="s">
-        <v>13</v>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2025-08-04</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>2.00% (+0.00%)</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>4.50% (+0.00%)</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>0.00% (-4.93%)</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>70.00% (+4.93%)</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>1.00% (+0.00%)</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>22.50% (+0.00%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2025-08-22</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>2.00% (+0.00%)</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>4.50% (+0.00%)</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>0.00% (+0.00%)</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>70.00% (+0.00%)</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>1.00% (+0.00%)</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>22.50% (+0.00%)</t>
+        </is>
       </c>
     </row>
   </sheetData>
@@ -519,9 +583,13 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:A1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
reset the config file and upload the empty report
</commit_message>
<xml_diff>
--- a/portfolio_summary.xlsx
+++ b/portfolio_summary.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Antho\Desktop\Git\portfolio_rebalance\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CB5E5917-B3AD-490F-9FDE-4B4E65D0D095}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0179A071-8E94-4B79-A750-0AEC51123E18}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="6120" yWindow="1695" windowWidth="14055" windowHeight="11295" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="rebalancing_overview" sheetId="1" r:id="rId1"/>
@@ -26,85 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="33">
-  <si>
-    <t>Rebalance_Date</t>
-  </si>
-  <si>
-    <t>AVDV</t>
-  </si>
-  <si>
-    <t>AVUV</t>
-  </si>
-  <si>
-    <t>CASH</t>
-  </si>
-  <si>
-    <t>SGOV</t>
-  </si>
-  <si>
-    <t>SQQQ</t>
-  </si>
-  <si>
-    <t>VT</t>
-  </si>
-  <si>
-    <t>2025-07-31</t>
-  </si>
-  <si>
-    <t>2.00% (+0.00%)</t>
-  </si>
-  <si>
-    <t>4.50% (+0.00%)</t>
-  </si>
-  <si>
-    <t>4.93% (+0.00%)</t>
-  </si>
-  <si>
-    <t>65.07% (+0.00%)</t>
-  </si>
-  <si>
-    <t>1.00% (+0.00%)</t>
-  </si>
-  <si>
-    <t>22.50% (+0.00%)</t>
-  </si>
-  <si>
-    <t>2025-08-04</t>
-  </si>
-  <si>
-    <t>0.00% (-4.93%)</t>
-  </si>
-  <si>
-    <t>70.00% (+4.93%)</t>
-  </si>
-  <si>
-    <t>2025-08-22</t>
-  </si>
-  <si>
-    <t>0.00% (+0.00%)</t>
-  </si>
-  <si>
-    <t>70.00% (+0.00%)</t>
-  </si>
-  <si>
-    <t>2025-10-13</t>
-  </si>
-  <si>
-    <t>0.00% (-2.00%)</t>
-  </si>
-  <si>
-    <t>0.00% (-4.50%)</t>
-  </si>
-  <si>
-    <t>5.00% (+5.00%)</t>
-  </si>
-  <si>
-    <t>0.00% (-1.00%)</t>
-  </si>
-  <si>
-    <t>25.00% (+2.50%)</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5" uniqueCount="5">
   <si>
     <t>report_gen_date</t>
   </si>
@@ -119,12 +41,6 @@
   </si>
   <si>
     <t>performance</t>
-  </si>
-  <si>
-    <t>4.40 (+3.31%)</t>
-  </si>
-  <si>
-    <t>-0.12 (-0.12%)</t>
   </si>
 </sst>
 </file>
@@ -487,17 +403,19 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G5"/>
+  <dimension ref="A1"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="1" width="15.42578125" bestFit="1" customWidth="1"/>
-    <col min="2" max="4" width="14.28515625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="15.28515625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="14.28515625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="15.28515625" bestFit="1" customWidth="1"/>
-  </cols>
+  <sheetData/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+  <dimension ref="A1:E1"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -513,165 +431,6 @@
       <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>7</v>
-      </c>
-      <c r="B2" t="s">
-        <v>8</v>
-      </c>
-      <c r="C2" t="s">
-        <v>9</v>
-      </c>
-      <c r="D2" t="s">
-        <v>10</v>
-      </c>
-      <c r="E2" t="s">
-        <v>11</v>
-      </c>
-      <c r="F2" t="s">
-        <v>12</v>
-      </c>
-      <c r="G2" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>14</v>
-      </c>
-      <c r="B3" t="s">
-        <v>8</v>
-      </c>
-      <c r="C3" t="s">
-        <v>9</v>
-      </c>
-      <c r="D3" t="s">
-        <v>15</v>
-      </c>
-      <c r="E3" t="s">
-        <v>16</v>
-      </c>
-      <c r="F3" t="s">
-        <v>12</v>
-      </c>
-      <c r="G3" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>17</v>
-      </c>
-      <c r="B4" t="s">
-        <v>8</v>
-      </c>
-      <c r="C4" t="s">
-        <v>9</v>
-      </c>
-      <c r="D4" t="s">
-        <v>18</v>
-      </c>
-      <c r="E4" t="s">
-        <v>19</v>
-      </c>
-      <c r="F4" t="s">
-        <v>12</v>
-      </c>
-      <c r="G4" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>20</v>
-      </c>
-      <c r="B5" t="s">
-        <v>21</v>
-      </c>
-      <c r="C5" t="s">
-        <v>22</v>
-      </c>
-      <c r="D5" t="s">
-        <v>23</v>
-      </c>
-      <c r="E5" t="s">
-        <v>19</v>
-      </c>
-      <c r="F5" t="s">
-        <v>24</v>
-      </c>
-      <c r="G5" t="s">
-        <v>25</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:E3"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>20</v>
-      </c>
-      <c r="B2" t="s">
-        <v>6</v>
-      </c>
-      <c r="C2">
-        <v>132.88</v>
-      </c>
-      <c r="D2">
-        <v>137.28</v>
-      </c>
-      <c r="E2" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>20</v>
-      </c>
-      <c r="B3" t="s">
-        <v>4</v>
-      </c>
-      <c r="C3">
-        <v>100.62</v>
-      </c>
-      <c r="D3">
-        <v>100.5</v>
-      </c>
-      <c r="E3" t="s">
-        <v>32</v>
-      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>